<commit_message>
removed gate pull down resistor and re-made erase and boot sequence of ESP32
</commit_message>
<xml_diff>
--- a/01_Hardware/BOM/BOM_V01.xlsx
+++ b/01_Hardware/BOM/BOM_V01.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="252">
   <si>
     <t xml:space="preserve">Reference</t>
   </si>
@@ -82,7 +82,7 @@
     <t xml:space="preserve">C102</t>
   </si>
   <si>
-    <t xml:space="preserve">100nF tantulum</t>
+    <t xml:space="preserve">100nF tantulum → 1uF</t>
   </si>
   <si>
     <t xml:space="preserve">Capacitor_SMD:C_1206_3216Metric</t>
@@ -380,6 +380,9 @@
   </si>
   <si>
     <t xml:space="preserve">Q101,Q102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">.</t>
   </si>
   <si>
     <t xml:space="preserve">STN3NF06L </t>
@@ -782,7 +785,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -806,6 +809,13 @@
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
@@ -825,7 +835,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -836,6 +846,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00A933"/>
+        <bgColor rgb="FF008000"/>
       </patternFill>
     </fill>
     <fill>
@@ -885,7 +901,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -898,35 +914,43 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -990,7 +1014,7 @@
       <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF00A933"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
@@ -1119,8 +1143,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="4.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="7.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="25.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="28.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="56.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="20.85"/>
@@ -1252,9 +1276,9 @@
         <v>5</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="F5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="5" t="s">
         <v>26</v>
       </c>
       <c r="G5" s="1" t="s">
@@ -1266,7 +1290,7 @@
       <c r="I5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" s="6" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1281,6 +1305,9 @@
         <f aca="false">B6*5</f>
         <v>10</v>
       </c>
+      <c r="D6" s="1" t="n">
+        <v>12</v>
+      </c>
       <c r="F6" s="1" t="s">
         <v>30</v>
       </c>
@@ -1308,6 +1335,9 @@
         <f aca="false">B7*5</f>
         <v>115</v>
       </c>
+      <c r="D7" s="1" t="n">
+        <v>220</v>
+      </c>
       <c r="F7" s="1" t="s">
         <v>35</v>
       </c>
@@ -1335,6 +1365,9 @@
         <f aca="false">B8*5</f>
         <v>20</v>
       </c>
+      <c r="D8" s="1" t="n">
+        <v>22</v>
+      </c>
       <c r="F8" s="1" t="s">
         <v>39</v>
       </c>
@@ -1362,6 +1395,9 @@
         <f aca="false">B9*5</f>
         <v>15</v>
       </c>
+      <c r="D9" s="1" t="n">
+        <v>20</v>
+      </c>
       <c r="F9" s="1" t="s">
         <v>39</v>
       </c>
@@ -1389,6 +1425,9 @@
         <f aca="false">B10*5</f>
         <v>5</v>
       </c>
+      <c r="D10" s="1" t="n">
+        <v>10</v>
+      </c>
       <c r="F10" s="1" t="s">
         <v>46</v>
       </c>
@@ -1416,6 +1455,9 @@
         <f aca="false">B11*5</f>
         <v>10</v>
       </c>
+      <c r="D11" s="1" t="n">
+        <v>12</v>
+      </c>
       <c r="F11" s="1" t="s">
         <v>14</v>
       </c>
@@ -1433,28 +1475,30 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B12" s="7" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="3" t="n">
         <f aca="false">B12*5</f>
         <v>10</v>
       </c>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5" t="s">
+      <c r="D12" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G12" s="7" t="s">
         <v>54</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="I12" s="6" t="s">
+      <c r="I12" s="8" t="s">
         <v>55</v>
       </c>
       <c r="J12" s="1" t="s">
@@ -1462,28 +1506,30 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B13" s="7" t="n">
         <v>2</v>
       </c>
       <c r="C13" s="3" t="n">
         <f aca="false">B13*5</f>
         <v>10</v>
       </c>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5" t="s">
+      <c r="D13" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="G13" s="7" t="s">
         <v>57</v>
       </c>
       <c r="H13" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="I13" s="6" t="s">
+      <c r="I13" s="8" t="s">
         <v>59</v>
       </c>
       <c r="J13" s="1" t="s">
@@ -1501,6 +1547,9 @@
         <f aca="false">B14*5</f>
         <v>5</v>
       </c>
+      <c r="D14" s="1" t="n">
+        <v>6</v>
+      </c>
       <c r="F14" s="1" t="s">
         <v>62</v>
       </c>
@@ -1528,6 +1577,9 @@
         <f aca="false">B15*5</f>
         <v>5</v>
       </c>
+      <c r="D15" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="F15" s="1" t="s">
         <v>66</v>
       </c>
@@ -1537,7 +1589,7 @@
       <c r="H15" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="I15" s="6" t="s">
+      <c r="I15" s="8" t="s">
         <v>67</v>
       </c>
       <c r="J15" s="1" t="s">
@@ -1555,6 +1607,9 @@
         <f aca="false">B16*5</f>
         <v>5</v>
       </c>
+      <c r="D16" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="F16" s="1" t="s">
         <v>46</v>
       </c>
@@ -1564,7 +1619,7 @@
       <c r="H16" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="I16" s="6" t="s">
+      <c r="I16" s="8" t="s">
         <v>70</v>
       </c>
       <c r="J16" s="1" t="s">
@@ -1582,6 +1637,9 @@
         <f aca="false">B17*5</f>
         <v>10</v>
       </c>
+      <c r="D17" s="1" t="n">
+        <v>20</v>
+      </c>
       <c r="F17" s="1" t="s">
         <v>73</v>
       </c>
@@ -1591,7 +1649,7 @@
       <c r="H17" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="I17" s="6" t="s">
+      <c r="I17" s="8" t="s">
         <v>74</v>
       </c>
       <c r="J17" s="1" t="s">
@@ -1599,24 +1657,24 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B18" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C18" s="8" t="n">
+      <c r="B18" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="10" t="n">
         <f aca="false">B18*5</f>
         <v>5</v>
       </c>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7" t="s">
+      <c r="D18" s="9"/>
+      <c r="E18" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="G18" s="7" t="s">
+      <c r="G18" s="9" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1631,6 +1689,9 @@
         <f aca="false">B19*5</f>
         <v>5</v>
       </c>
+      <c r="D19" s="1" t="n">
+        <v>10</v>
+      </c>
       <c r="F19" s="1" t="s">
         <v>79</v>
       </c>
@@ -1640,7 +1701,7 @@
       <c r="H19" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="I19" s="6" t="s">
+      <c r="I19" s="8" t="s">
         <v>82</v>
       </c>
       <c r="J19" s="1" t="s">
@@ -1658,6 +1719,9 @@
         <f aca="false">B20*5</f>
         <v>35</v>
       </c>
+      <c r="D20" s="1" t="n">
+        <v>40</v>
+      </c>
       <c r="F20" s="1" t="s">
         <v>85</v>
       </c>
@@ -1667,7 +1731,7 @@
       <c r="H20" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="I20" s="6" t="s">
+      <c r="I20" s="8" t="s">
         <v>88</v>
       </c>
       <c r="J20" s="1" t="s">
@@ -1685,6 +1749,9 @@
         <f aca="false">B21*5</f>
         <v>15</v>
       </c>
+      <c r="D21" s="1" t="n">
+        <v>20</v>
+      </c>
       <c r="F21" s="1" t="s">
         <v>91</v>
       </c>
@@ -1708,7 +1775,7 @@
       <c r="B22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C22" s="9" t="n">
+      <c r="C22" s="11" t="n">
         <f aca="false">B22*5</f>
         <v>5</v>
       </c>
@@ -1728,7 +1795,7 @@
       <c r="B23" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C23" s="9" t="n">
+      <c r="C23" s="11" t="n">
         <f aca="false">B23*5</f>
         <v>5</v>
       </c>
@@ -1752,6 +1819,9 @@
         <f aca="false">B24*5</f>
         <v>5</v>
       </c>
+      <c r="D24" s="1" t="n">
+        <v>6</v>
+      </c>
       <c r="F24" s="1" t="s">
         <v>102</v>
       </c>
@@ -1819,6 +1889,9 @@
         <f aca="false">B27*5</f>
         <v>5</v>
       </c>
+      <c r="D27" s="1" t="n">
+        <v>5</v>
+      </c>
       <c r="F27" s="1" t="s">
         <v>114</v>
       </c>
@@ -1828,7 +1901,7 @@
       <c r="H27" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="I27" s="6" t="s">
+      <c r="I27" s="8" t="s">
         <v>117</v>
       </c>
       <c r="J27" s="1" t="s">
@@ -1842,29 +1915,31 @@
       <c r="B28" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C28" s="3" t="n">
-        <f aca="false">B28*5</f>
-        <v>10</v>
+      <c r="C28" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>12</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G28" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I28" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="H28" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>120</v>
-      </c>
       <c r="J28" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B29" s="1" t="n">
         <v>4</v>
@@ -1873,25 +1948,28 @@
         <f aca="false">B29*5</f>
         <v>20</v>
       </c>
+      <c r="D29" s="1" t="n">
+        <v>40</v>
+      </c>
       <c r="F29" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="I29" s="6" t="s">
         <v>128</v>
       </c>
+      <c r="I29" s="8" t="s">
+        <v>129</v>
+      </c>
       <c r="J29" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B30" s="1" t="n">
         <v>3</v>
@@ -1900,25 +1978,28 @@
         <f aca="false">B30*5</f>
         <v>15</v>
       </c>
+      <c r="D30" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="F30" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H30" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="I30" s="6" t="s">
-        <v>132</v>
+      <c r="I30" s="8" t="s">
+        <v>133</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B31" s="1" t="n">
         <v>2</v>
@@ -1927,25 +2008,28 @@
         <f aca="false">B31*5</f>
         <v>10</v>
       </c>
+      <c r="D31" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="F31" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="I31" s="6" t="s">
         <v>138</v>
       </c>
+      <c r="I31" s="8" t="s">
+        <v>139</v>
+      </c>
       <c r="J31" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B32" s="1" t="n">
         <v>1</v>
@@ -1954,25 +2038,28 @@
         <f aca="false">B32*5</f>
         <v>5</v>
       </c>
+      <c r="D32" s="1" t="n">
+        <v>10</v>
+      </c>
       <c r="F32" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B33" s="1" t="n">
         <v>8</v>
@@ -1981,25 +2068,28 @@
         <f aca="false">B33*5</f>
         <v>40</v>
       </c>
+      <c r="D33" s="1" t="n">
+        <v>50</v>
+      </c>
       <c r="F33" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="I33" s="6" t="s">
         <v>150</v>
       </c>
+      <c r="I33" s="8" t="s">
+        <v>151</v>
+      </c>
       <c r="J33" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B34" s="1" t="n">
         <v>15</v>
@@ -2008,25 +2098,28 @@
         <f aca="false">B34*5</f>
         <v>75</v>
       </c>
+      <c r="D34" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="F34" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="I34" s="6" t="s">
-        <v>154</v>
+        <v>150</v>
+      </c>
+      <c r="I34" s="8" t="s">
+        <v>155</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B35" s="1" t="n">
         <v>1</v>
@@ -2035,25 +2128,28 @@
         <f aca="false">B35*5</f>
         <v>5</v>
       </c>
+      <c r="D35" s="1" t="n">
+        <v>7</v>
+      </c>
       <c r="F35" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H35" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="6" t="s">
-        <v>158</v>
+      <c r="I35" s="8" t="s">
+        <v>159</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B36" s="1" t="n">
         <v>1</v>
@@ -2062,25 +2158,28 @@
         <f aca="false">B36*5</f>
         <v>5</v>
       </c>
+      <c r="D36" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="F36" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H36" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="6" t="s">
-        <v>162</v>
+      <c r="I36" s="8" t="s">
+        <v>163</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B37" s="1" t="n">
         <v>1</v>
@@ -2089,25 +2188,28 @@
         <f aca="false">B37*5</f>
         <v>5</v>
       </c>
+      <c r="D37" s="1" t="n">
+        <v>60</v>
+      </c>
       <c r="F37" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B38" s="1" t="n">
         <v>12</v>
@@ -2116,25 +2218,28 @@
         <f aca="false">B38*5</f>
         <v>60</v>
       </c>
+      <c r="D38" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="F38" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="I38" s="6" t="s">
-        <v>171</v>
+        <v>150</v>
+      </c>
+      <c r="I38" s="8" t="s">
+        <v>172</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B39" s="1" t="n">
         <v>1</v>
@@ -2143,25 +2248,28 @@
         <f aca="false">B39*5</f>
         <v>5</v>
       </c>
+      <c r="D39" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="F39" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B40" s="1" t="n">
         <v>10</v>
@@ -2170,25 +2278,28 @@
         <f aca="false">B40*5</f>
         <v>50</v>
       </c>
+      <c r="D40" s="1" t="n">
+        <v>200</v>
+      </c>
       <c r="F40" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="I40" s="6" t="s">
-        <v>179</v>
+        <v>150</v>
+      </c>
+      <c r="I40" s="8" t="s">
+        <v>180</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B41" s="1" t="n">
         <v>3</v>
@@ -2197,25 +2308,28 @@
         <f aca="false">B41*5</f>
         <v>15</v>
       </c>
+      <c r="D41" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="F41" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="I41" s="6" t="s">
-        <v>183</v>
+        <v>150</v>
+      </c>
+      <c r="I41" s="8" t="s">
+        <v>184</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B42" s="1" t="n">
         <v>1</v>
@@ -2224,47 +2338,50 @@
         <f aca="false">B42*5</f>
         <v>5</v>
       </c>
+      <c r="D42" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="F42" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H42" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="I42" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="J42" s="1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="B43" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" s="10" t="n">
+        <f aca="false">B43*5</f>
+        <v>5</v>
+      </c>
+      <c r="D43" s="9"/>
+      <c r="E43" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="G43" s="9" t="s">
         <v>149</v>
-      </c>
-      <c r="I42" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="J42" s="1" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="B43" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C43" s="8" t="n">
-        <f aca="false">B43*5</f>
-        <v>5</v>
-      </c>
-      <c r="D43" s="7"/>
-      <c r="E43" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="F43" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="G43" s="7" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B44" s="1" t="n">
         <v>1</v>
@@ -2273,25 +2390,28 @@
         <f aca="false">B44*5</f>
         <v>5</v>
       </c>
+      <c r="D44" s="1" t="n">
+        <v>20</v>
+      </c>
       <c r="F44" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="I44" s="6" t="s">
-        <v>192</v>
+        <v>150</v>
+      </c>
+      <c r="I44" s="8" t="s">
+        <v>193</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B45" s="1" t="n">
         <v>5</v>
@@ -2300,25 +2420,28 @@
         <f aca="false">B45*5</f>
         <v>25</v>
       </c>
+      <c r="D45" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="F45" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="I45" s="6" t="s">
-        <v>196</v>
+        <v>150</v>
+      </c>
+      <c r="I45" s="8" t="s">
+        <v>197</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B46" s="1" t="n">
         <v>3</v>
@@ -2327,25 +2450,28 @@
         <f aca="false">B46*5</f>
         <v>15</v>
       </c>
+      <c r="D46" s="1" t="n">
+        <v>20</v>
+      </c>
       <c r="F46" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="I46" s="6" t="s">
-        <v>200</v>
+        <v>150</v>
+      </c>
+      <c r="I46" s="8" t="s">
+        <v>201</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B47" s="1" t="n">
         <v>2</v>
@@ -2354,25 +2480,28 @@
         <f aca="false">B47*5</f>
         <v>10</v>
       </c>
+      <c r="D47" s="1" t="n">
+        <v>12</v>
+      </c>
       <c r="F47" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="I47" s="6" t="s">
         <v>206</v>
       </c>
+      <c r="I47" s="8" t="s">
+        <v>207</v>
+      </c>
       <c r="J47" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B48" s="1" t="n">
         <v>1</v>
@@ -2381,25 +2510,28 @@
         <f aca="false">B48*5</f>
         <v>5</v>
       </c>
+      <c r="D48" s="1" t="n">
+        <v>5</v>
+      </c>
       <c r="F48" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J48" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B49" s="1" t="n">
         <v>1</v>
@@ -2408,25 +2540,28 @@
         <f aca="false">B49*5</f>
         <v>5</v>
       </c>
+      <c r="D49" s="1" t="n">
+        <v>5</v>
+      </c>
       <c r="F49" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="I49" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J49" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B50" s="1" t="n">
         <v>1</v>
@@ -2435,25 +2570,28 @@
         <f aca="false">B50*5</f>
         <v>5</v>
       </c>
+      <c r="D50" s="1" t="n">
+        <v>5</v>
+      </c>
       <c r="F50" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>224</v>
-      </c>
-      <c r="J50" s="10" t="s">
         <v>225</v>
+      </c>
+      <c r="J50" s="12" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B51" s="1" t="n">
         <v>1</v>
@@ -2462,25 +2600,28 @@
         <f aca="false">B51*5</f>
         <v>5</v>
       </c>
+      <c r="D51" s="1" t="n">
+        <v>5</v>
+      </c>
       <c r="F51" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B52" s="1" t="n">
         <v>1</v>
@@ -2489,25 +2630,28 @@
         <f aca="false">B52*5</f>
         <v>5</v>
       </c>
+      <c r="D52" s="1" t="n">
+        <v>5</v>
+      </c>
       <c r="F52" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="J52" s="10" t="s">
         <v>235</v>
+      </c>
+      <c r="J52" s="12" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B53" s="1" t="n">
         <v>1</v>
@@ -2516,25 +2660,28 @@
         <f aca="false">B53*5</f>
         <v>5</v>
       </c>
+      <c r="D53" s="1" t="n">
+        <v>5</v>
+      </c>
       <c r="F53" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>1</v>
@@ -2546,24 +2693,24 @@
       <c r="D54" s="2"/>
       <c r="E54" s="2"/>
       <c r="F54" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>1</v>
@@ -2575,16 +2722,17 @@
       <c r="D55" s="2"/>
       <c r="E55" s="2"/>
       <c r="F55" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="J50" r:id="rId1" display="https://www.mouser.it/ProductDetail/Espressif-Systems/ESP32-WROOM-32E-N8?qs=sGAEpiMZZMu3sxpa5v1qrkR%2F6t0IkXq84gmxxC8jME0%3D"/>
-    <hyperlink ref="J52" r:id="rId2" display="https://www.mouser.it/ProductDetail/STMicroelectronics/USBLC6-2P6?qs=6ARB0lp6jlViGcbUSvj1Mw%3D%3D"/>
+    <hyperlink ref="J5" r:id="rId1" display="https://www.mouser.it/ProductDetail/KEMET/T491A106K016AT7280?qs=WOKUqv%2F%2FT%2FYL9FI%252BTlhIbw%3D%3D"/>
+    <hyperlink ref="J50" r:id="rId2" display="https://www.mouser.it/ProductDetail/Espressif-Systems/ESP32-WROOM-32E-N8?qs=sGAEpiMZZMu3sxpa5v1qrkR%2F6t0IkXq84gmxxC8jME0%3D"/>
+    <hyperlink ref="J52" r:id="rId3" display="https://www.mouser.it/ProductDetail/STMicroelectronics/USBLC6-2P6?qs=6ARB0lp6jlViGcbUSvj1Mw%3D%3D"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>